<commit_message>
the fight exe is be packed but i cna't guarantee if there are any other libraries being packaged in
</commit_message>
<xml_diff>
--- a/WTF-Trans/output.xlsx
+++ b/WTF-Trans/output.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -534,7 +534,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2025-05-27</t>
+          <t>2025-05-30</t>
         </is>
       </c>
       <c r="I2" t="inlineStr"/>
@@ -594,7 +594,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2025-05-27</t>
+          <t>2025-05-30</t>
         </is>
       </c>
       <c r="I3" t="inlineStr"/>
@@ -654,7 +654,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2025-05-27</t>
+          <t>2025-05-30</t>
         </is>
       </c>
       <c r="I4" t="inlineStr"/>
@@ -714,7 +714,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2025-05-27</t>
+          <t>2025-05-30</t>
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
@@ -774,7 +774,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2025-05-27</t>
+          <t>2025-05-30</t>
         </is>
       </c>
       <c r="I6" t="inlineStr"/>
@@ -834,7 +834,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2025-05-27</t>
+          <t>2025-05-30</t>
         </is>
       </c>
       <c r="I7" t="inlineStr"/>
@@ -894,7 +894,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2025-05-27</t>
+          <t>2025-05-30</t>
         </is>
       </c>
       <c r="I8" t="inlineStr"/>
@@ -954,7 +954,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2025-05-27</t>
+          <t>2025-05-30</t>
         </is>
       </c>
       <c r="I9" t="inlineStr"/>
@@ -1014,7 +1014,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2025-05-27</t>
+          <t>2025-05-30</t>
         </is>
       </c>
       <c r="I10" t="inlineStr"/>
@@ -1074,7 +1074,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2025-05-27</t>
+          <t>2025-05-30</t>
         </is>
       </c>
       <c r="I11" t="inlineStr"/>
@@ -1134,7 +1134,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2025-05-27</t>
+          <t>2025-05-30</t>
         </is>
       </c>
       <c r="I12" t="inlineStr"/>
@@ -1194,7 +1194,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2025-05-27</t>
+          <t>2025-05-30</t>
         </is>
       </c>
       <c r="I13" t="inlineStr"/>
@@ -1254,7 +1254,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2025-05-27</t>
+          <t>2025-05-30</t>
         </is>
       </c>
       <c r="I14" t="inlineStr"/>
@@ -1314,7 +1314,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2025-05-27</t>
+          <t>2025-05-30</t>
         </is>
       </c>
       <c r="I15" t="inlineStr"/>
@@ -1374,7 +1374,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2025-05-27</t>
+          <t>2025-05-30</t>
         </is>
       </c>
       <c r="I16" t="inlineStr"/>
@@ -1434,7 +1434,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2025-05-27</t>
+          <t>2025-05-30</t>
         </is>
       </c>
       <c r="I17" t="inlineStr"/>
@@ -1490,7 +1490,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2025-05-27</t>
+          <t>2025-05-30</t>
         </is>
       </c>
       <c r="I18" t="inlineStr"/>
@@ -1542,7 +1542,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2025-05-27</t>
+          <t>2025-05-30</t>
         </is>
       </c>
       <c r="I19" t="inlineStr"/>
@@ -1598,7 +1598,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2025-05-27</t>
+          <t>2025-05-30</t>
         </is>
       </c>
       <c r="I20" t="inlineStr"/>
@@ -1650,7 +1650,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2025-05-27</t>
+          <t>2025-05-30</t>
         </is>
       </c>
       <c r="I21" t="inlineStr"/>
@@ -1706,7 +1706,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>2025-05-27</t>
+          <t>2025-05-30</t>
         </is>
       </c>
       <c r="I22" t="inlineStr"/>
@@ -1762,7 +1762,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>2025-05-27</t>
+          <t>2025-05-30</t>
         </is>
       </c>
       <c r="I23" t="inlineStr"/>
@@ -1818,7 +1818,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>2025-05-27</t>
+          <t>2025-05-30</t>
         </is>
       </c>
       <c r="I24" t="inlineStr"/>
@@ -1874,7 +1874,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>2025-05-27</t>
+          <t>2025-05-30</t>
         </is>
       </c>
       <c r="I25" t="inlineStr"/>
@@ -1930,7 +1930,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>2025-05-27</t>
+          <t>2025-05-30</t>
         </is>
       </c>
       <c r="I26" t="inlineStr"/>
@@ -1986,7 +1986,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>2025-05-27</t>
+          <t>2025-05-30</t>
         </is>
       </c>
       <c r="I27" t="inlineStr"/>
@@ -2042,7 +2042,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>2025-05-27</t>
+          <t>2025-05-30</t>
         </is>
       </c>
       <c r="I28" t="inlineStr"/>
@@ -2102,7 +2102,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>2025-05-27</t>
+          <t>2025-05-30</t>
         </is>
       </c>
       <c r="I29" t="inlineStr"/>
@@ -2158,7 +2158,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>2025-05-27</t>
+          <t>2025-05-30</t>
         </is>
       </c>
       <c r="I30" t="inlineStr"/>
@@ -2218,7 +2218,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>2025-05-27</t>
+          <t>2025-05-30</t>
         </is>
       </c>
       <c r="I31" t="inlineStr"/>
@@ -2274,7 +2274,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>2025-05-27</t>
+          <t>2025-05-30</t>
         </is>
       </c>
       <c r="I32" t="inlineStr"/>
@@ -2334,7 +2334,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>2025-05-27</t>
+          <t>2025-05-30</t>
         </is>
       </c>
       <c r="I33" t="inlineStr"/>
@@ -2394,7 +2394,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>2025-05-27</t>
+          <t>2025-05-30</t>
         </is>
       </c>
       <c r="I34" t="inlineStr"/>
@@ -2454,7 +2454,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>2025-05-27</t>
+          <t>2025-05-30</t>
         </is>
       </c>
       <c r="I35" t="inlineStr"/>
@@ -2514,7 +2514,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>2025-05-27</t>
+          <t>2025-05-30</t>
         </is>
       </c>
       <c r="I36" t="inlineStr"/>
@@ -2574,7 +2574,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>2025-05-27</t>
+          <t>2025-05-30</t>
         </is>
       </c>
       <c r="I37" t="inlineStr"/>
@@ -2634,7 +2634,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>2025-05-27</t>
+          <t>2025-05-30</t>
         </is>
       </c>
       <c r="I38" t="inlineStr"/>
@@ -2694,7 +2694,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>2025-05-27</t>
+          <t>2025-05-30</t>
         </is>
       </c>
       <c r="I39" t="inlineStr"/>
@@ -2754,7 +2754,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>2025-05-27</t>
+          <t>2025-05-30</t>
         </is>
       </c>
       <c r="I40" t="inlineStr"/>
@@ -2799,7 +2799,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2040</t>
+          <t>1040</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2814,7 +2814,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>2025-05-28</t>
+          <t>2025-05-30</t>
         </is>
       </c>
       <c r="I41" t="inlineStr"/>

</xml_diff>